<commit_message>
notas projeto UniRuy Wyden todas
</commit_message>
<xml_diff>
--- a/05 Others/2026.1 Avaliação Projetos/Turma Engenharia de Software - ARA0097 Turma 3002  PRESENCIAL Wyden UniRuy 2026_1.xlsx
+++ b/05 Others/2026.1 Avaliação Projetos/Turma Engenharia de Software - ARA0097 Turma 3002  PRESENCIAL Wyden UniRuy 2026_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\Avaliações Yduqs 2022_2 BDQ 2023_1 2024_2\2026.1 Avaliação Projetos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B59B27-9D26-4EFA-970D-3029EB8DFEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D193E4D2-AE65-4B40-BCA7-A57DEA01C420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD6ED3E7-57DF-4A52-9E4C-63B0F7661B3D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="55">
   <si>
     <t>Falta</t>
   </si>
@@ -147,6 +147,61 @@
   </si>
   <si>
     <t>SSA, 05 de JUNHO de 2026</t>
+  </si>
+  <si>
+    <t>EQ</t>
+  </si>
+  <si>
+    <t>https://github.com/aryaneandrade/projeto-monitorias-uniruy</t>
+  </si>
+  <si>
+    <t>https://github.com/imthedavi/iFrango</t>
+  </si>
+  <si>
+    <t>https://github.com/EricAssisdev/FACULDADE/tree/main/EngenhariaDeSoftware/TrabalhoEngSoft</t>
+  </si>
+  <si>
+    <t>https://github.com/JoaoVictorCarvalho-DEV/trabalho_arquitetura_de_software</t>
+  </si>
+  <si>
+    <t>https://github.com/Raymond-slayer/FACULDADE/tree/main/EngenhariaDeSoftware/TrabalhoEngSoft</t>
+  </si>
+  <si>
+    <t>https://github.com/diaszin/trabalho-final-engenharia-de-software-uniruy</t>
+  </si>
+  <si>
+    <t>https://github.com/PnpmGK/PROJETO-VESTURE</t>
+  </si>
+  <si>
+    <t>https://github.com/1LeoAlves/D.O.M.E-Project</t>
+  </si>
+  <si>
+    <t>https://github.com/MajuGoes/CineBR_Engenharia_Software</t>
+  </si>
+  <si>
+    <t>https://github.com/machadorenata119-del/Projeto-de-Engenharia-de-software-</t>
+  </si>
+  <si>
+    <t>https://github.com/Rodrigoo2006/Projeto-Monitorias</t>
+  </si>
+  <si>
+    <t>https://github.com/YanAugusto2031/TaurusFit</t>
+  </si>
+  <si>
+    <t>VSSTickets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/vitorsantanauniruy/Engenharia_software_apresenta-o
+</t>
+  </si>
+  <si>
+    <t>https://engenharia-software-apresenta-o.vercel.app/</t>
+  </si>
+  <si>
+    <t>não GitHub; somente PPT</t>
+  </si>
+  <si>
+    <t>Não fez</t>
   </si>
 </sst>
 </file>
@@ -156,7 +211,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,8 +245,22 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,8 +273,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -387,12 +468,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -406,41 +538,96 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
@@ -774,808 +961,953 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0212B8F-44EC-4B38-84EB-21D2846DA7CB}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="84.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="13">
-        <v>0</v>
-      </c>
-      <c r="C2" s="13">
-        <v>0</v>
-      </c>
-      <c r="D2" s="14">
+      <c r="B2" s="14">
+        <v>4</v>
+      </c>
+      <c r="C2" s="11">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11">
+        <v>0</v>
+      </c>
+      <c r="E2" s="12">
         <v>0.9</v>
       </c>
-      <c r="E2" s="14">
+      <c r="F2" s="12">
         <v>0.4</v>
       </c>
-      <c r="F2" s="13">
-        <f>$B$2/7*4</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="13">
-        <v>0</v>
-      </c>
-      <c r="H2" s="13">
-        <f>F2+G2</f>
-        <v>0</v>
-      </c>
-      <c r="I2" s="15"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G2" s="11">
+        <f>$C$2/7*4</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="11">
+        <v>6</v>
+      </c>
+      <c r="I2" s="11">
+        <f>G2+H2</f>
+        <v>6</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="4">
-        <v>0</v>
+      <c r="B3" s="15">
+        <v>5</v>
       </c>
       <c r="C3" s="4">
         <v>0</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0.4</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>0.7</v>
       </c>
-      <c r="F3" s="4">
-        <f>$B$2/7*4</f>
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
+        <f>$C$2/7*4</f>
         <v>0</v>
       </c>
       <c r="H3" s="4">
-        <f>F3+G3</f>
-        <v>0</v>
-      </c>
-      <c r="I3" s="7"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="4">
+        <f>G3+H3</f>
+        <v>6</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
-        <v>0</v>
-      </c>
+      <c r="B4" s="17"/>
       <c r="C4" s="4">
         <v>0</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0.7</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <f t="shared" ref="F4:F27" si="0">$B$2/7*4</f>
+      <c r="F4" s="5" t="s">
         <v>0</v>
       </c>
       <c r="G4" s="4">
+        <f t="shared" ref="G4:G27" si="0">$C$2/7*4</f>
         <v>0</v>
       </c>
       <c r="H4" s="4">
-        <f t="shared" ref="H4:H27" si="1">F4+G4</f>
-        <v>0</v>
-      </c>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I4" s="18">
+        <f t="shared" ref="I4:I27" si="1">G4+H4</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4">
-        <v>0</v>
+      <c r="B5" s="15">
+        <v>10</v>
       </c>
       <c r="C5" s="4">
         <v>0</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0.5</v>
       </c>
-      <c r="E5" s="5">
+      <c r="F5" s="5">
         <v>0.9</v>
       </c>
-      <c r="F5" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H5" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="7"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B6" s="27"/>
+      <c r="C6" s="28">
+        <v>0</v>
+      </c>
+      <c r="D6" s="28">
+        <v>0</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="28">
+        <v>0</v>
+      </c>
+      <c r="I6" s="30">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="4">
-        <v>0</v>
-      </c>
+      <c r="B7" s="15"/>
       <c r="C7" s="4">
         <v>0</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
         <v>1</v>
       </c>
-      <c r="E7" s="5">
+      <c r="F7" s="5">
         <v>0.6</v>
       </c>
-      <c r="F7" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H7" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4">
-        <v>0</v>
+      <c r="B8" s="15">
+        <v>1</v>
       </c>
       <c r="C8" s="4">
         <v>0</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5">
         <v>0.6</v>
       </c>
-      <c r="E8" s="5">
+      <c r="F8" s="5">
         <v>0.8</v>
       </c>
-      <c r="F8" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J8" s="21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="4">
-        <v>0</v>
-      </c>
+      <c r="B9" s="15"/>
       <c r="C9" s="4">
         <v>0</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5">
         <v>0.6</v>
       </c>
-      <c r="E9" s="5">
+      <c r="F9" s="5">
         <v>0.5</v>
       </c>
-      <c r="F9" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H9" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="7"/>
+    </row>
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="4">
-        <v>0</v>
+      <c r="B10" s="15">
+        <v>3</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5">
         <v>0.7</v>
       </c>
-      <c r="E10" s="5">
+      <c r="F10" s="5">
         <v>0.6</v>
       </c>
-      <c r="F10" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="4">
-        <v>0</v>
+      <c r="B11" s="15">
+        <v>6</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
         <v>0.9</v>
       </c>
-      <c r="E11" s="5">
+      <c r="F11" s="5">
         <v>0.5</v>
       </c>
-      <c r="F11" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H11" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="7"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+      <c r="I11" s="4">
+        <f t="shared" si="1"/>
+        <v>4.5</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="4">
-        <v>0</v>
+      <c r="B12" s="15">
+        <v>1</v>
       </c>
       <c r="C12" s="4">
         <v>0</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
         <v>0.6</v>
       </c>
-      <c r="E12" s="5">
+      <c r="F12" s="5">
         <v>0.4</v>
       </c>
-      <c r="F12" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I12" s="7"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="I12" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J12" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="4">
-        <v>0</v>
+      <c r="B13" s="15">
+        <v>2</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
         <v>0.7</v>
       </c>
-      <c r="E13" s="5">
+      <c r="F13" s="5">
         <v>0.6</v>
       </c>
-      <c r="F13" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="7"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="I13" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="4">
-        <v>0</v>
+      <c r="B14" s="15">
+        <v>4</v>
       </c>
       <c r="C14" s="4">
         <v>0</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
         <v>0.4</v>
       </c>
-      <c r="E14" s="5">
+      <c r="F14" s="5">
         <v>0.5</v>
       </c>
-      <c r="F14" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="7"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I14" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="4">
-        <v>0</v>
-      </c>
+      <c r="B15" s="15"/>
       <c r="C15" s="4">
         <v>0</v>
       </c>
-      <c r="D15" s="5">
-        <v>0.9</v>
+      <c r="D15" s="4">
+        <v>0</v>
       </c>
       <c r="E15" s="5">
         <v>0.9</v>
       </c>
-      <c r="F15" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="F15" s="5">
+        <v>0.9</v>
       </c>
       <c r="G15" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="4">
-        <v>0</v>
-      </c>
+      <c r="B16" s="15"/>
       <c r="C16" s="4">
         <v>0</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
         <v>0.8</v>
       </c>
-      <c r="E16" s="5">
+      <c r="F16" s="5">
         <v>0.6</v>
       </c>
-      <c r="F16" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="4">
-        <v>0</v>
+      <c r="B17" s="15">
+        <v>3</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
         <v>0.5</v>
       </c>
-      <c r="E17" s="5">
+      <c r="F17" s="5">
         <v>0.3</v>
       </c>
-      <c r="F17" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I17" s="7"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="I17" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="4">
-        <v>0</v>
+      <c r="B18" s="15">
+        <v>2</v>
       </c>
       <c r="C18" s="4">
         <v>0</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5">
         <v>0.6</v>
       </c>
-      <c r="E18" s="5">
+      <c r="F18" s="5">
         <v>0.4</v>
       </c>
-      <c r="F18" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="I18" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J18" s="21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="4">
-        <v>0</v>
+      <c r="B19" s="15">
+        <v>3</v>
       </c>
       <c r="C19" s="4">
         <v>0</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5">
         <v>0.4</v>
       </c>
-      <c r="E19" s="5">
+      <c r="F19" s="5">
         <v>0.2</v>
       </c>
-      <c r="F19" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I19" s="7"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="I19" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J19" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="4">
-        <v>0</v>
+      <c r="B20" s="15">
+        <v>5</v>
       </c>
       <c r="C20" s="4">
         <v>0</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
         <v>0.6</v>
       </c>
-      <c r="E20" s="5">
+      <c r="F20" s="5">
         <v>0.5</v>
       </c>
-      <c r="F20" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I20" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="4">
-        <v>0</v>
-      </c>
+      <c r="B21" s="17"/>
       <c r="C21" s="4">
         <v>0</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="4">
         <v>0</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F21" s="4">
-        <f t="shared" si="0"/>
+      <c r="F21" s="5" t="s">
         <v>0</v>
       </c>
       <c r="G21" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="I21" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="25"/>
+    </row>
+    <row r="22" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="4">
-        <v>0</v>
+      <c r="B22" s="15">
+        <v>4</v>
       </c>
       <c r="C22" s="4">
         <v>0</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
         <v>0.9</v>
       </c>
-      <c r="E22" s="5">
+      <c r="F22" s="5">
         <v>0.3</v>
       </c>
-      <c r="F22" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="7"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="J22" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="4">
-        <v>0</v>
+      <c r="B23" s="15">
+        <v>14</v>
       </c>
       <c r="C23" s="4">
         <v>0</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5">
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
         <v>0.4</v>
       </c>
-      <c r="F23" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I23" s="7"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="4">
-        <v>0</v>
+      <c r="B24" s="15">
+        <v>10</v>
       </c>
       <c r="C24" s="4">
         <v>0</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
         <v>0.6</v>
       </c>
-      <c r="E24" s="5">
+      <c r="F24" s="5">
         <v>0.4</v>
       </c>
-      <c r="F24" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I24" s="7"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="4">
-        <v>0</v>
+      <c r="B25" s="15">
+        <v>9</v>
       </c>
       <c r="C25" s="4">
         <v>0</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="4">
         <v>0</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F25" s="4">
-        <f t="shared" si="0"/>
+      <c r="F25" s="5" t="s">
         <v>0</v>
       </c>
       <c r="G25" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I25" s="7"/>
-    </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J25" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="4">
-        <v>0</v>
+      <c r="B26" s="15">
+        <v>15</v>
       </c>
       <c r="C26" s="4">
         <v>0</v>
       </c>
-      <c r="D26" s="5">
-        <v>0.8</v>
+      <c r="D26" s="4">
+        <v>0</v>
       </c>
       <c r="E26" s="5">
         <v>0.8</v>
       </c>
-      <c r="F26" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="F26" s="5">
+        <v>0.8</v>
       </c>
       <c r="G26" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I26" s="7"/>
-    </row>
-    <row r="27" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="I26" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J26" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="K26" t="s">
+        <v>50</v>
+      </c>
+      <c r="L26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="9">
-        <v>0</v>
-      </c>
-      <c r="C27" s="9">
-        <v>0</v>
-      </c>
-      <c r="D27" s="10">
+      <c r="B27" s="16">
+        <v>9</v>
+      </c>
+      <c r="C27" s="8">
+        <v>0</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0</v>
+      </c>
+      <c r="E27" s="9">
         <v>0.8</v>
       </c>
-      <c r="E27" s="10">
+      <c r="F27" s="9">
         <v>0.9</v>
       </c>
-      <c r="F27" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G27" s="9">
-        <v>0</v>
-      </c>
-      <c r="H27" s="9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I27" s="11"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G27" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="8">
+        <v>0</v>
+      </c>
+      <c r="I27" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="24" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J5" r:id="rId1" xr:uid="{64307761-D7D9-4A06-8E9B-6432284E854E}"/>
+    <hyperlink ref="J7" r:id="rId2" xr:uid="{9FF9BA28-8CB3-4B80-8505-0DD5A4B4E98B}"/>
+    <hyperlink ref="J8" r:id="rId3" xr:uid="{5B4F64D5-2DB4-482B-95DD-80B3761005D1}"/>
+    <hyperlink ref="J10" r:id="rId4" xr:uid="{BE74226B-EF15-4116-B4F1-19B8C5FA7A05}"/>
+    <hyperlink ref="J12" r:id="rId5" xr:uid="{DE7AC3EA-4613-4AC4-B20A-90FA62B313AE}"/>
+    <hyperlink ref="J14" r:id="rId6" xr:uid="{D7F6D36F-6A10-4B7A-AA02-E6C9E6B5C051}"/>
+    <hyperlink ref="J16" r:id="rId7" xr:uid="{0737A2F4-2758-4383-9AC6-554918D8AAD2}"/>
+    <hyperlink ref="J17" r:id="rId8" xr:uid="{7CE1E1A0-7FCD-425F-9410-F078CFFA05F5}"/>
+    <hyperlink ref="J18" r:id="rId9" xr:uid="{BA41D141-0138-4C5C-A3D9-4BF95A26BC3D}"/>
+    <hyperlink ref="J19" r:id="rId10" xr:uid="{53AAE598-84E9-4C79-9E24-CA2C883B6E66}"/>
+    <hyperlink ref="J23" r:id="rId11" xr:uid="{79A6158E-E06C-4AC2-A309-D77F5EED1094}"/>
+    <hyperlink ref="J24" r:id="rId12" xr:uid="{FD5ED851-BE40-4735-855D-CF806D52DAAA}"/>
+    <hyperlink ref="J27" r:id="rId13" xr:uid="{0463F0AB-72AD-4F0A-B0CA-15B47959AB87}"/>
+    <hyperlink ref="J25" r:id="rId14" xr:uid="{EFE5979B-08C9-4CE0-8148-D0A1E6738E3A}"/>
+    <hyperlink ref="J15" r:id="rId15" xr:uid="{8EC7AABD-09D1-478A-B9AC-83E277E6B4AA}"/>
+    <hyperlink ref="J22" r:id="rId16" xr:uid="{3056A8A1-666B-456E-B9F5-99383D083EC4}"/>
+    <hyperlink ref="J2" r:id="rId17" xr:uid="{DCAB900F-B8B1-4E77-A5F0-93EC30C1F226}"/>
+    <hyperlink ref="J26" r:id="rId18" xr:uid="{C1FB3950-AE45-460B-8E7D-5534614908AA}"/>
+    <hyperlink ref="J3" r:id="rId19" xr:uid="{B8D6459A-3387-4805-8DCE-1592045B4C97}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>